<commit_message>
paper run 2026-09-24 11:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-24.xlsx
+++ b/reports/2026-09-24.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -724,13 +724,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>152.72</v>
+        <v>278.4</v>
       </c>
       <c r="E15" t="n">
         <v>8.279999999999999</v>
@@ -743,13 +743,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>66.23999999999999</v>
+        <v>339.97</v>
       </c>
       <c r="E16" t="n">
         <v>49.44</v>
@@ -765,107 +765,119 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>147.38</v>
+        <v>54.94</v>
       </c>
       <c r="E18" t="n">
-        <v>49.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>71.58</v>
+        <v>234.3</v>
       </c>
       <c r="E19" t="n">
-        <v>8.279999999999999</v>
+        <v>49.44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>329.13</v>
+      </c>
+      <c r="E20" t="n">
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>152.72</v>
-      </c>
-      <c r="E21" t="n">
-        <v>8.279999999999999</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>66.23999999999999</v>
+        <v>310.38</v>
       </c>
       <c r="E22" t="n">
-        <v>49.44</v>
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>197.48</v>
+      </c>
+      <c r="E23" t="n">
+        <v>49.44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>81.14</v>
+        <v>110.51</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -874,318 +886,344 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>2</v>
-      </c>
-      <c r="C25" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" t="n">
-        <v>137.82</v>
-      </c>
-      <c r="E25" t="n">
-        <v>57.72</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>7</v>
+      </c>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" t="n">
+        <v>480.55</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>137.82</v>
+      </c>
+      <c r="E27" t="n">
+        <v>57.72</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>49.44</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>8.279999999999999</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>49.44</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="n">
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>8.279999999999999</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>49.44</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>8.279999999999999</v>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>49.44</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
-        <v>49.44</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>8.279999999999999</v>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>49.44</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>49.44</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>49.44</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>2</v>
-      </c>
-      <c r="C46" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" t="n">
-        <v>57.72</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>57.72</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B51" t="n">
         <v>2</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C51" t="n">
         <v>2</v>
       </c>
-      <c r="D49" t="n">
+      <c r="D51" t="n">
         <v>57.72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-09-24 17:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-24.xlsx
+++ b/reports/2026-09-24.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,49 @@
       </c>
       <c r="K3" t="n">
         <v>49.44</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-24T17:13:45.898647+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00141</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>8.4</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -633,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57.72</v>
+        <v>66.12</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>57.72</v>
+        <v>66.12</v>
       </c>
     </row>
     <row r="8">
@@ -673,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1738.420000000001</v>
+        <v>1746.820000000001</v>
       </c>
     </row>
     <row r="12">
@@ -724,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>278.4</v>
+        <v>157.34</v>
       </c>
       <c r="E15" t="n">
         <v>8.279999999999999</v>
@@ -743,16 +786,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>339.97</v>
+        <v>692.13</v>
       </c>
       <c r="E16" t="n">
-        <v>49.44</v>
+        <v>57.84</v>
       </c>
     </row>
     <row r="17">
@@ -784,447 +827,482 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>234.3</v>
+        <v>-86.92</v>
       </c>
       <c r="E19" t="n">
-        <v>49.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>329.13</v>
+        <v>480.89</v>
       </c>
       <c r="E20" t="n">
-        <v>8.279999999999999</v>
+        <v>57.84</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>9</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" t="n">
+        <v>400.56</v>
+      </c>
+      <c r="E21" t="n">
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>4</v>
-      </c>
-      <c r="C22" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" t="n">
-        <v>310.38</v>
-      </c>
-      <c r="E22" t="n">
-        <v>8.279999999999999</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
-        <v>197.48</v>
+        <v>216.78</v>
       </c>
       <c r="E23" t="n">
-        <v>49.44</v>
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>110.51</v>
+        <v>426.43</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>57.84</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>206.26</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>7</v>
-      </c>
-      <c r="C26" t="n">
-        <v>7</v>
-      </c>
-      <c r="D26" t="n">
-        <v>480.55</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>15</v>
+      </c>
+      <c r="C27" t="n">
+        <v>13</v>
+      </c>
+      <c r="D27" t="n">
+        <v>653.74</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" t="n">
-        <v>137.82</v>
-      </c>
-      <c r="E27" t="n">
-        <v>57.72</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>195.73</v>
+      </c>
+      <c r="E28" t="n">
+        <v>66.12</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>49.44</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>57.84</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>XRP</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
         <v>8.279999999999999</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>8.279999999999999</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>8.279999999999999</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>49.44</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>57.84</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>8.279999999999999</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>8.279999999999999</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
         <v>49.44</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" t="n">
-        <v>8.279999999999999</v>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>8.4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" t="n">
-        <v>49.44</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8.279999999999999</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>57.84</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>2</v>
-      </c>
-      <c r="C48" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" t="n">
-        <v>57.72</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>66.12</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="n">
-        <v>57.72</v>
+      <c r="B53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>66.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-24 23:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-24.xlsx
+++ b/reports/2026-09-24.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,49 @@
       </c>
       <c r="K4" t="n">
         <v>8.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-24T21:58:22.168155+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.6011</v>
+      </c>
+      <c r="F5" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>103.64</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00159</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>-62.3</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -656,7 +699,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -666,7 +709,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6">
@@ -676,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66.12</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="7">
@@ -696,7 +739,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-62.3</v>
       </c>
     </row>
     <row r="9">
@@ -706,7 +749,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1746.820000000001</v>
+        <v>1684.520000000001</v>
       </c>
     </row>
     <row r="12">
@@ -767,16 +810,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>157.34</v>
+        <v>64.51000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>8.279999999999999</v>
+        <v>-54.02</v>
       </c>
     </row>
     <row r="16">
@@ -869,16 +912,16 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>12</v>
+      </c>
+      <c r="C21" t="n">
         <v>9</v>
       </c>
-      <c r="C21" t="n">
-        <v>8</v>
-      </c>
       <c r="D21" t="n">
-        <v>400.56</v>
+        <v>307.73</v>
       </c>
       <c r="E21" t="n">
-        <v>8.279999999999999</v>
+        <v>-54.02</v>
       </c>
     </row>
     <row r="22">
@@ -895,13 +938,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>216.78</v>
+        <v>288.52</v>
       </c>
       <c r="E23" t="n">
         <v>8.279999999999999</v>
@@ -914,13 +957,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
         <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>426.43</v>
+        <v>349.2</v>
       </c>
       <c r="E24" t="n">
         <v>57.84</v>
@@ -933,16 +976,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" t="n">
         <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>206.26</v>
+        <v>118.92</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-62.3</v>
       </c>
     </row>
     <row r="26">
@@ -959,13 +1002,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D27" t="n">
-        <v>653.74</v>
+        <v>648.25</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -978,16 +1021,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C28" t="n">
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>195.73</v>
+        <v>108.39</v>
       </c>
       <c r="E28" t="n">
-        <v>66.12</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="30">
@@ -1042,13 +1085,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>8.279999999999999</v>
+        <v>-54.02</v>
       </c>
     </row>
     <row r="36">
@@ -1080,13 +1123,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
         <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>8.279999999999999</v>
+        <v>-54.02</v>
       </c>
     </row>
     <row r="38">
@@ -1175,134 +1218,198 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-62.3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
-        <v>8.279999999999999</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>8.279999999999999</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>0.55–0.60</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B48" t="n">
         <v>2</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C48" t="n">
         <v>2</v>
       </c>
-      <c r="D47" t="n">
+      <c r="D48" t="n">
         <v>57.84</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-62.3</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>3</v>
-      </c>
-      <c r="C50" t="n">
-        <v>3</v>
-      </c>
-      <c r="D50" t="n">
-        <v>66.12</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
+        <v>66.12</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-62.3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B56" t="n">
         <v>3</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C56" t="n">
         <v>3</v>
       </c>
-      <c r="D53" t="n">
+      <c r="D56" t="n">
         <v>66.12</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-62.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>